<commit_message>
Normalise line endings, commit plan updates
.gitattributes stores every text file with LF and marks the Office
files binary so they are never line-ending converted.

Also commits the working changes to Plan.xlsx, Proposal.docx and
Research.xlsx.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Research.xlsx
+++ b/Research.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VSF\Project INFO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VSF\Project 4week\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19980CA4-C9AB-4EFA-A124-01722159265F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5E0B3472-9DC8-4102-A7FF-0260799D13A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1815" yWindow="1905" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tổng quan nội bộ" sheetId="1" r:id="rId1"/>
@@ -1388,7 +1388,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K199"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -1402,7 +1402,7 @@
     <col min="11" max="11" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.95" customHeight="1">
+    <row r="1" spans="1:11" ht="27.9" customHeight="1">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -1417,7 +1417,7 @@
     <row r="2" spans="1:11">
       <c r="A2" s="4"/>
     </row>
-    <row r="3" spans="1:11" ht="15">
+    <row r="3" spans="1:11">
       <c r="A3" s="11" t="s">
         <v>1</v>
       </c>
@@ -1427,7 +1427,7 @@
       <c r="J3" s="12"/>
       <c r="K3" s="12"/>
     </row>
-    <row r="4" spans="1:11" ht="28.5">
+    <row r="4" spans="1:11" ht="27.6">
       <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
@@ -1466,7 +1466,7 @@
     <row r="8" spans="1:11">
       <c r="A8" s="4"/>
     </row>
-    <row r="9" spans="1:11" ht="30">
+    <row r="9" spans="1:11" ht="27.6">
       <c r="A9" s="11" t="s">
         <v>9</v>
       </c>
@@ -1492,7 +1492,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="71.25">
+    <row r="10" spans="1:11" ht="69">
       <c r="A10" s="6" t="s">
         <v>17</v>
       </c>
@@ -1518,7 +1518,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="85.5">
+    <row r="11" spans="1:11" ht="82.8">
       <c r="A11" s="6" t="s">
         <v>25</v>
       </c>
@@ -1544,7 +1544,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="42.75">
+    <row r="12" spans="1:11" ht="41.4">
       <c r="A12" s="6" t="s">
         <v>32</v>
       </c>
@@ -1570,7 +1570,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="42.75">
+    <row r="13" spans="1:11" ht="41.4">
       <c r="A13" s="6" t="s">
         <v>39</v>
       </c>
@@ -1596,7 +1596,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="42.75">
+    <row r="14" spans="1:11" ht="41.4">
       <c r="A14" s="6" t="s">
         <v>46</v>
       </c>
@@ -1622,7 +1622,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="42.75">
+    <row r="15" spans="1:11" ht="41.4">
       <c r="A15" s="6" t="s">
         <v>54</v>
       </c>
@@ -1648,7 +1648,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="42.75">
+    <row r="16" spans="1:11" ht="41.4">
       <c r="A16" s="6" t="s">
         <v>62</v>
       </c>
@@ -1674,7 +1674,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="42.75">
+    <row r="17" spans="1:8" ht="41.4">
       <c r="A17" s="8" t="s">
         <v>69</v>
       </c>
@@ -2260,7 +2260,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G200"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="4" width="34" customWidth="1"/>
@@ -2269,7 +2269,7 @@
     <col min="7" max="7" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="27.95" customHeight="1">
+    <row r="1" spans="1:7" ht="27.9" customHeight="1">
       <c r="A1" s="13" t="s">
         <v>76</v>
       </c>
@@ -2283,7 +2283,7 @@
     <row r="2" spans="1:7">
       <c r="A2" s="4"/>
     </row>
-    <row r="3" spans="1:7" ht="30">
+    <row r="3" spans="1:7" ht="27.6">
       <c r="A3" s="11" t="s">
         <v>77</v>
       </c>
@@ -2306,7 +2306,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="85.5">
+    <row r="4" spans="1:7" ht="82.8">
       <c r="A4" s="6" t="s">
         <v>84</v>
       </c>
@@ -2329,7 +2329,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="71.25">
+    <row r="5" spans="1:7" ht="69">
       <c r="A5" s="6" t="s">
         <v>90</v>
       </c>
@@ -2352,7 +2352,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="28.5">
+    <row r="6" spans="1:7" ht="27.6">
       <c r="A6" s="6" t="s">
         <v>95</v>
       </c>
@@ -2375,7 +2375,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="85.5">
+    <row r="7" spans="1:7" ht="82.8">
       <c r="A7" s="6" t="s">
         <v>102</v>
       </c>
@@ -2398,7 +2398,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="114">
+    <row r="8" spans="1:7" ht="96.6">
       <c r="A8" s="8" t="s">
         <v>108</v>
       </c>
@@ -3011,7 +3011,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H200"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="38" customWidth="1"/>
@@ -3023,7 +3023,7 @@
     <col min="8" max="8" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="27.95" customHeight="1">
+    <row r="1" spans="1:8" ht="27.9" customHeight="1">
       <c r="A1" s="13" t="s">
         <v>115</v>
       </c>
@@ -3038,7 +3038,7 @@
     <row r="2" spans="1:8">
       <c r="A2" s="4"/>
     </row>
-    <row r="3" spans="1:8" ht="15">
+    <row r="3" spans="1:8">
       <c r="A3" s="11" t="s">
         <v>116</v>
       </c>
@@ -3064,7 +3064,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="42.75">
+    <row r="4" spans="1:8" ht="41.4">
       <c r="A4" s="6" t="s">
         <v>123</v>
       </c>
@@ -3090,7 +3090,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="28.5">
+    <row r="5" spans="1:8" ht="27.6">
       <c r="A5" s="6" t="s">
         <v>130</v>
       </c>
@@ -3116,7 +3116,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="42.75">
+    <row r="6" spans="1:8" ht="41.4">
       <c r="A6" s="6" t="s">
         <v>136</v>
       </c>
@@ -3142,7 +3142,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="28.5">
+    <row r="7" spans="1:8" ht="27.6">
       <c r="A7" s="6" t="s">
         <v>142</v>
       </c>
@@ -3168,7 +3168,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="42.75">
+    <row r="8" spans="1:8" ht="41.4">
       <c r="A8" s="6" t="s">
         <v>148</v>
       </c>
@@ -3194,7 +3194,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="42.75">
+    <row r="9" spans="1:8" ht="41.4">
       <c r="A9" s="8" t="s">
         <v>154</v>
       </c>
@@ -3807,7 +3807,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H199"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
@@ -3819,7 +3819,7 @@
     <col min="8" max="8" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="27.95" customHeight="1">
+    <row r="1" spans="1:8" ht="27.9" customHeight="1">
       <c r="A1" s="13" t="s">
         <v>159</v>
       </c>
@@ -3834,7 +3834,7 @@
     <row r="2" spans="1:8">
       <c r="A2" s="4"/>
     </row>
-    <row r="3" spans="1:8" ht="15">
+    <row r="3" spans="1:8">
       <c r="A3" s="11" t="s">
         <v>160</v>
       </c>
@@ -3860,7 +3860,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="42.75">
+    <row r="4" spans="1:8" ht="41.4">
       <c r="A4" s="6" t="s">
         <v>167</v>
       </c>
@@ -3886,7 +3886,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="42.75">
+    <row r="5" spans="1:8" ht="41.4">
       <c r="A5" s="6" t="s">
         <v>175</v>
       </c>
@@ -3912,7 +3912,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="28.5">
+    <row r="6" spans="1:8" ht="27.6">
       <c r="A6" s="6" t="s">
         <v>182</v>
       </c>
@@ -3938,7 +3938,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="28.5">
+    <row r="7" spans="1:8" ht="27.6">
       <c r="A7" s="8" t="s">
         <v>189</v>
       </c>
@@ -4554,7 +4554,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:H200"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="3" width="18" customWidth="1"/>
@@ -4564,7 +4564,7 @@
     <col min="7" max="8" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="27.95" customHeight="1">
+    <row r="1" spans="1:8" ht="27.9" customHeight="1">
       <c r="A1" s="13" t="s">
         <v>306</v>
       </c>
@@ -4579,7 +4579,7 @@
     <row r="2" spans="1:8">
       <c r="A2" s="4"/>
     </row>
-    <row r="3" spans="1:8" ht="15">
+    <row r="3" spans="1:8">
       <c r="A3" s="11" t="s">
         <v>196</v>
       </c>
@@ -4605,7 +4605,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="28.5">
+    <row r="4" spans="1:8" ht="27.6">
       <c r="A4" s="6" t="s">
         <v>204</v>
       </c>
@@ -4631,7 +4631,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15">
+    <row r="5" spans="1:8">
       <c r="A5" s="6" t="s">
         <v>84</v>
       </c>
@@ -4657,7 +4657,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15">
+    <row r="6" spans="1:8">
       <c r="A6" s="6" t="s">
         <v>214</v>
       </c>
@@ -4683,7 +4683,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="28.5">
+    <row r="7" spans="1:8" ht="27.6">
       <c r="A7" s="6" t="s">
         <v>220</v>
       </c>
@@ -4709,7 +4709,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15">
+    <row r="8" spans="1:8">
       <c r="A8" s="6" t="s">
         <v>225</v>
       </c>
@@ -4735,7 +4735,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="28.5">
+    <row r="9" spans="1:8" ht="27.6">
       <c r="A9" s="6" t="s">
         <v>230</v>
       </c>
@@ -4761,7 +4761,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="15">
+    <row r="10" spans="1:8">
       <c r="A10" s="6" t="s">
         <v>235</v>
       </c>
@@ -4787,7 +4787,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="15">
+    <row r="11" spans="1:8">
       <c r="A11" s="6" t="s">
         <v>240</v>
       </c>
@@ -4813,7 +4813,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="15">
+    <row r="12" spans="1:8">
       <c r="A12" s="6" t="s">
         <v>32</v>
       </c>
@@ -4839,7 +4839,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="15">
+    <row r="13" spans="1:8">
       <c r="A13" s="6" t="s">
         <v>249</v>
       </c>
@@ -4865,7 +4865,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="28.5">
+    <row r="14" spans="1:8" ht="27.6">
       <c r="A14" s="6" t="s">
         <v>253</v>
       </c>
@@ -4891,7 +4891,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="15">
+    <row r="15" spans="1:8">
       <c r="A15" s="6" t="s">
         <v>46</v>
       </c>
@@ -4917,7 +4917,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="15">
+    <row r="16" spans="1:8">
       <c r="A16" s="6" t="s">
         <v>262</v>
       </c>
@@ -4943,7 +4943,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="28.5">
+    <row r="17" spans="1:8" ht="27.6">
       <c r="A17" s="6" t="s">
         <v>266</v>
       </c>
@@ -4969,7 +4969,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="15">
+    <row r="18" spans="1:8">
       <c r="A18" s="6" t="s">
         <v>272</v>
       </c>
@@ -4995,7 +4995,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="28.5">
+    <row r="19" spans="1:8" ht="27.6">
       <c r="A19" s="6" t="s">
         <v>276</v>
       </c>
@@ -5021,7 +5021,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="28.5">
+    <row r="20" spans="1:8" ht="27.6">
       <c r="A20" s="6" t="s">
         <v>282</v>
       </c>
@@ -5047,7 +5047,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="15">
+    <row r="21" spans="1:8">
       <c r="A21" s="6" t="s">
         <v>288</v>
       </c>
@@ -5073,7 +5073,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="15">
+    <row r="22" spans="1:8">
       <c r="A22" s="6" t="s">
         <v>292</v>
       </c>
@@ -5099,7 +5099,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="28.5">
+    <row r="23" spans="1:8" ht="27.6">
       <c r="A23" s="6" t="s">
         <v>297</v>
       </c>
@@ -5125,7 +5125,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="28.5">
+    <row r="24" spans="1:8" ht="27.6">
       <c r="A24" s="8" t="s">
         <v>301</v>
       </c>

</xml_diff>